<commit_message>
fix: replace tutorial contacts and exclude runtime artifacts from releases
</commit_message>
<xml_diff>
--- a/FHD/frontend/public/tutorial/xcagi-quickstart-sample-b.xlsx
+++ b/FHD/frontend/public/tutorial/xcagi-quickstart-sample-b.xlsx
@@ -46,8 +46,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -122,6 +123,26 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>XCMAX</author>
+  </authors>
+  <commentList>
+    <comment ref="C2" authorId="0" shapeId="0">
+      <text>
+        <t>合成教程占位值：11个0，不可拨号，不代表真实联系人。</t>
+      </text>
+    </comment>
+    <comment ref="C3" authorId="0" shapeId="0">
+      <text>
+        <t>合成教程占位值：11个0，不可拨号，不代表真实联系人。</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -436,38 +457,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>教程示例-张三</t>
+          <t>教程示例-虚构联系人甲</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>市场部</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>13800000001</t>
+          <t>教程示例-部门甲</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>00000000000</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>教程示例-李四</t>
+          <t>教程示例-虚构联系人乙</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>研发部</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>13800000002</t>
+          <t>教程示例-部门乙</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>00000000000</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>